<commit_message>
fix(budget): adjust total funding request to strict BAYLAT 8.000 EUR ceiling
</commit_message>
<xml_diff>
--- a/06_Reiseverwaltung_Kostenkalkulation_Anschubfinanzierung.xlsx
+++ b/06_Reiseverwaltung_Kostenkalkulation_Anschubfinanzierung.xlsx
@@ -1759,7 +1759,7 @@
       </c>
       <c r="B25" s="19" t="n"/>
       <c r="C25" s="102" t="n">
-        <v>5765</v>
+        <v>5205</v>
       </c>
       <c r="G25" s="77" t="n"/>
     </row>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="C35" s="102" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="36" ht="5.1" customFormat="1" customHeight="1" s="39" thickBot="1" thickTop="1"/>
@@ -1897,11 +1897,11 @@
     <col width="15.5703125" customWidth="1" style="39" min="6" max="6"/>
     <col width="12.28515625" customWidth="1" style="41" min="7" max="7"/>
     <col width="16.28515625" customWidth="1" style="41" min="8" max="8"/>
-    <col hidden="1" style="39" min="9" max="9"/>
+    <col hidden="1" width="13" customWidth="1" style="39" min="9" max="9"/>
     <col hidden="1" width="10.7109375" customWidth="1" style="39" min="10" max="10"/>
     <col hidden="1" width="4.28515625" customWidth="1" style="39" min="11" max="11"/>
     <col hidden="1" width="12.28515625" customWidth="1" style="39" min="12" max="12"/>
-    <col hidden="1" style="39" min="13" max="313"/>
+    <col hidden="1" width="13" customWidth="1" style="39" min="13" max="313"/>
     <col width="20.140625" customWidth="1" style="39" min="314" max="314"/>
     <col width="10.85546875" customWidth="1" style="39" min="315" max="16384"/>
   </cols>
@@ -2170,10 +2170,10 @@
         </is>
       </c>
       <c r="G13" s="111" t="n">
-        <v>1600</v>
+        <v>1450</v>
       </c>
       <c r="H13" s="111" t="n">
-        <v>1600</v>
+        <v>1450</v>
       </c>
       <c r="I13" s="58" t="n"/>
       <c r="K13" s="65" t="inlineStr">
@@ -2322,10 +2322,10 @@
         </is>
       </c>
       <c r="G17" s="115" t="n">
-        <v>1700</v>
+        <v>1500</v>
       </c>
       <c r="H17" s="115" t="n">
-        <v>1700</v>
+        <v>1500</v>
       </c>
       <c r="I17" s="58" t="n"/>
       <c r="M17" s="49" t="n">
@@ -2346,7 +2346,7 @@
       <c r="D18" s="114" t="n"/>
       <c r="E18" s="70" t="inlineStr">
         <is>
-          <t>21 Übernachtungen in Deggendorf/Passau, je Nacht 65 Euro</t>
+          <t>21 Übernachtungen in Deggendorf/Passau, je Nacht 55 Euro</t>
         </is>
       </c>
       <c r="F18" s="63" t="inlineStr">
@@ -2355,10 +2355,10 @@
         </is>
       </c>
       <c r="G18" s="115" t="n">
-        <v>1365</v>
+        <v>1155</v>
       </c>
       <c r="H18" s="115" t="n">
-        <v>1365</v>
+        <v>1155</v>
       </c>
       <c r="M18" s="49" t="n">
         <v>2028</v>
@@ -2471,7 +2471,7 @@
       <c r="D22" s="114" t="n"/>
       <c r="E22" s="70" t="inlineStr">
         <is>
-          <t>Zubehör und Sachkosten für hybride Workshop-Übertragung und Datenintegration</t>
+          <t>Zubehör und Sachkosten für hybride Workshop-Übertragung und Datenintegration (anteilig)</t>
         </is>
       </c>
       <c r="F22" s="63" t="inlineStr">
@@ -2480,10 +2480,10 @@
         </is>
       </c>
       <c r="G22" s="115" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H22" s="115" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="LB22" s="18" t="n"/>
     </row>

</xml_diff>

<commit_message>
refactor(scientific-proposal): academic overhaul of Spanish exposé, OASys and budget synchronization
- Restructured expose_propuesta_cientifica_baylat_es.typ into 8 formal scientific sections
- Preserved Table 4.1 Benchmark and eliminated AI clichés and neural loss math
- Adjusted Deggendorf stay duration to strictly 2 weeks (14 days / 14 nights)
- Synchronized budget across Spanish exposé, OASys, and Excel to 7.350 € (<= 8.000 €)
- Expanded references.bib with 30 authoritative citations (FNC, SCA, AOAC, ISO, 2018-2026 literature)
- Verified 100% pass across all 3 adversarial and regression test suites
</commit_message>
<xml_diff>
--- a/06_Reiseverwaltung_Kostenkalkulation_Anschubfinanzierung.xlsx
+++ b/06_Reiseverwaltung_Kostenkalkulation_Anschubfinanzierung.xlsx
@@ -1759,7 +1759,7 @@
       </c>
       <c r="B25" s="19" t="n"/>
       <c r="C25" s="102" t="n">
-        <v>5205</v>
+        <v>4820</v>
       </c>
       <c r="G25" s="77" t="n"/>
     </row>
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="C27" s="102" t="n">
-        <v>1445</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="28" ht="5.1" customFormat="1" customHeight="1" s="39" thickBot="1" thickTop="1">
@@ -1800,7 +1800,7 @@
         </is>
       </c>
       <c r="C31" s="102" t="n">
-        <v>400</v>
+        <v>450</v>
       </c>
     </row>
     <row r="32" ht="5.1" customFormat="1" customHeight="1" s="39" thickBot="1" thickTop="1">
@@ -2284,10 +2284,10 @@
         </is>
       </c>
       <c r="G16" s="115" t="n">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="H16" s="115" t="n">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="I16" s="58" t="n"/>
       <c r="K16" s="65" t="inlineStr">
@@ -2346,7 +2346,7 @@
       <c r="D18" s="114" t="n"/>
       <c r="E18" s="70" t="inlineStr">
         <is>
-          <t>21 Übernachtungen in Deggendorf/Passau, je Nacht 55 Euro</t>
+          <t>14 Übernachtungen in Deggendorf/Passau, je Nacht 55 Euro</t>
         </is>
       </c>
       <c r="F18" s="63" t="inlineStr">
@@ -2355,10 +2355,10 @@
         </is>
       </c>
       <c r="G18" s="115" t="n">
-        <v>1155</v>
+        <v>770</v>
       </c>
       <c r="H18" s="115" t="n">
-        <v>1155</v>
+        <v>770</v>
       </c>
       <c r="M18" s="49" t="n">
         <v>2028</v>
@@ -2378,7 +2378,7 @@
       <c r="D19" s="114" t="n"/>
       <c r="E19" s="70" t="inlineStr">
         <is>
-          <t>21 Tage Tagegeldpauschale Deutschland (gem. BayRKG/DAAD), je 45 Euro pro Tag</t>
+          <t>14 Tage Tagegeldpauschale Deutschland (gem. BayRKG/DAAD), je 45 Euro pro Tag</t>
         </is>
       </c>
       <c r="F19" s="63" t="inlineStr">
@@ -2387,10 +2387,10 @@
         </is>
       </c>
       <c r="G19" s="115" t="n">
-        <v>945</v>
+        <v>630</v>
       </c>
       <c r="H19" s="115" t="n">
-        <v>945</v>
+        <v>630</v>
       </c>
       <c r="M19" s="49" t="n">
         <v>2029</v>

</xml_diff>

<commit_message>
feat: actualizacion de titulo global y traduccion completa del expose en ingles
</commit_message>
<xml_diff>
--- a/06_Reiseverwaltung_Kostenkalkulation_Anschubfinanzierung.xlsx
+++ b/06_Reiseverwaltung_Kostenkalkulation_Anschubfinanzierung.xlsx
@@ -1701,7 +1701,7 @@
       </c>
       <c r="B16" s="96" t="inlineStr">
         <is>
-          <t>Physik-informierte neuronale Differentialgleichungen und multimodale Spektralsensorik zur autonomen Qualitäts- und Frischevorhersage von kolumbianischem Spezialitätenkaffee</t>
+          <t>Künstliche Intelligenz und Spektroskopie zur Bewertung der Lebensmittelqualität</t>
         </is>
       </c>
       <c r="C16" s="97" t="n"/>
@@ -2060,7 +2060,7 @@
       <c r="C10" s="50" t="n"/>
       <c r="D10" s="52" t="inlineStr">
         <is>
-          <t>Physik-informierte neuronale Differentialgleichungen und multimodale Spektralsensorik (Spezialitätenkaffee)</t>
+          <t>Künstliche Intelligenz und Spektroskopie zur Bewertung der Lebensmittelqualität</t>
         </is>
       </c>
       <c r="E10" s="104" t="n"/>

</xml_diff>